<commit_message>
fix: distribucion desigual de ventas por asesor en Q4 2025 (antes 3-3-3-3-3, ahora con ranking real)
- 26 negocios Ganado en vez de 15, repartidos sin uniformidad: Luis Bedoya 8, Sofia Prada 6, Ana Quintero 5, Miguel Salazar 4, Paula Arenas 3
- Permite identificar un top vendedor real en vez de un empate artificial
- Proyectos y Financiero actualizados en consecuencia (26 pagos iniciales nuevos)

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/database/CRM_Inmobiliario_DLOGIA.xlsx
+++ b/database/CRM_Inmobiliario_DLOGIA.xlsx
@@ -640,13 +640,13 @@
         <v>120</v>
       </c>
       <c r="G3" s="6" t="n">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="H3" s="6" t="n">
         <v>15</v>
       </c>
       <c r="I3" s="6" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="J3" s="6" t="n">
         <v>9500000</v>
@@ -687,13 +687,13 @@
         <v>60</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="H4" s="9" t="n">
         <v>8</v>
       </c>
       <c r="I4" s="9" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J4" s="9" t="n">
         <v>6800000</v>
@@ -734,13 +734,13 @@
         <v>200</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="H5" s="6" t="n">
         <v>22</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="J5" s="6" t="n">
         <v>7200000</v>
@@ -828,13 +828,13 @@
         <v>150</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="H7" s="6" t="n">
         <v>30</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="J7" s="6" t="n">
         <v>4800000</v>
@@ -875,13 +875,13 @@
         <v>40</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H8" s="9" t="n">
         <v>5</v>
       </c>
       <c r="I8" s="9" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J8" s="9" t="n">
         <v>8100000</v>
@@ -4790,7 +4790,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L57"/>
+  <dimension ref="A1:L68"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="12" customWidth="1" style="25" min="1" max="1"/>
@@ -7140,7 +7140,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Ana Quintero</t>
+          <t>Luis Bedoya</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -7149,19 +7149,19 @@
         </is>
       </c>
       <c r="G43" t="n">
-        <v>620000000</v>
+        <v>705000000</v>
       </c>
       <c r="H43" t="n">
         <v>1</v>
       </c>
       <c r="I43" s="27" t="n">
-        <v>45894</v>
+        <v>45889</v>
       </c>
       <c r="J43" s="27" t="n">
-        <v>45938</v>
+        <v>45935</v>
       </c>
       <c r="K43" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="L43" t="inlineStr">
         <is>
@@ -7201,19 +7201,19 @@
         </is>
       </c>
       <c r="G44" t="n">
-        <v>705000000</v>
+        <v>640000000</v>
       </c>
       <c r="H44" t="n">
         <v>1</v>
       </c>
       <c r="I44" s="27" t="n">
-        <v>45910</v>
+        <v>45905</v>
       </c>
       <c r="J44" s="27" t="n">
-        <v>45952</v>
+        <v>45950</v>
       </c>
       <c r="K44" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="L44" t="inlineStr">
         <is>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Tomás Escobar</t>
+          <t>Ricardo Palacio</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -7239,12 +7239,12 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Apto 302</t>
+          <t>Apto 1102</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Paula Arenas</t>
+          <t>Luis Bedoya</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -7259,13 +7259,13 @@
         <v>1</v>
       </c>
       <c r="I45" s="27" t="n">
-        <v>45922</v>
+        <v>45931</v>
       </c>
       <c r="J45" s="27" t="n">
-        <v>45966</v>
+        <v>45976</v>
       </c>
       <c r="K45" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="L45" t="inlineStr">
         <is>
@@ -7281,7 +7281,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Melissa Uribe</t>
+          <t>Tomás Escobar</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -7296,7 +7296,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Sofía Prada</t>
+          <t>Luis Bedoya</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -7305,19 +7305,19 @@
         </is>
       </c>
       <c r="G46" t="n">
-        <v>640000000</v>
+        <v>610000000</v>
       </c>
       <c r="H46" t="n">
         <v>1</v>
       </c>
       <c r="I46" s="27" t="n">
-        <v>45901</v>
+        <v>45915</v>
       </c>
       <c r="J46" s="27" t="n">
-        <v>45945</v>
+        <v>45958</v>
       </c>
       <c r="K46" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="L46" t="inlineStr">
         <is>
@@ -7333,7 +7333,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Andrés Zuluaga</t>
+          <t>Melissa Uribe</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -7348,7 +7348,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Miguel Salazar</t>
+          <t>Luis Bedoya</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -7357,19 +7357,19 @@
         </is>
       </c>
       <c r="G47" t="n">
-        <v>590000000</v>
+        <v>555000000</v>
       </c>
       <c r="H47" t="n">
         <v>1</v>
       </c>
       <c r="I47" s="27" t="n">
-        <v>45935</v>
+        <v>45940</v>
       </c>
       <c r="J47" s="27" t="n">
-        <v>45980</v>
+        <v>45983</v>
       </c>
       <c r="K47" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="L47" t="inlineStr">
         <is>
@@ -7385,7 +7385,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Paula Betancur</t>
+          <t>Andrés Zuluaga</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -7400,7 +7400,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Ana Quintero</t>
+          <t>Luis Bedoya</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -7409,16 +7409,16 @@
         </is>
       </c>
       <c r="G48" t="n">
-        <v>540000000</v>
+        <v>545000000</v>
       </c>
       <c r="H48" t="n">
         <v>1</v>
       </c>
       <c r="I48" s="27" t="n">
-        <v>45914</v>
+        <v>45920</v>
       </c>
       <c r="J48" s="27" t="n">
-        <v>45957</v>
+        <v>45963</v>
       </c>
       <c r="K48" t="n">
         <v>43</v>
@@ -7437,7 +7437,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Camilo Restrepo</t>
+          <t>Paula Betancur</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -7461,19 +7461,19 @@
         </is>
       </c>
       <c r="G49" t="n">
-        <v>610000000</v>
+        <v>615000000</v>
       </c>
       <c r="H49" t="n">
         <v>1</v>
       </c>
       <c r="I49" s="27" t="n">
-        <v>45928</v>
+        <v>45955</v>
       </c>
       <c r="J49" s="27" t="n">
-        <v>45973</v>
+        <v>45999</v>
       </c>
       <c r="K49" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="L49" t="inlineStr">
         <is>
@@ -7489,22 +7489,22 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Sara Londoño</t>
+          <t>Camilo Restrepo</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>PRY-003</t>
+          <t>PRY-006</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Apto 675</t>
+          <t>Apto 460</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Miguel Salazar</t>
+          <t>Luis Bedoya</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -7513,19 +7513,19 @@
         </is>
       </c>
       <c r="G50" t="n">
-        <v>560000000</v>
+        <v>470000000</v>
       </c>
       <c r="H50" t="n">
         <v>1</v>
       </c>
       <c r="I50" s="27" t="n">
-        <v>45950</v>
+        <v>45960</v>
       </c>
       <c r="J50" s="27" t="n">
-        <v>45994</v>
+        <v>46003</v>
       </c>
       <c r="K50" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="L50" t="inlineStr">
         <is>
@@ -7541,22 +7541,22 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Julián Osorio</t>
+          <t>Sara Londoño</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>PRY-005</t>
+          <t>PRY-001</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Apto 322</t>
+          <t>Apto 302</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Ana Quintero</t>
+          <t>Sofía Prada</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -7565,19 +7565,19 @@
         </is>
       </c>
       <c r="G51" t="n">
-        <v>460000000</v>
+        <v>690000000</v>
       </c>
       <c r="H51" t="n">
         <v>1</v>
       </c>
       <c r="I51" s="27" t="n">
-        <v>45905</v>
+        <v>45901</v>
       </c>
       <c r="J51" s="27" t="n">
-        <v>45950</v>
+        <v>45944</v>
       </c>
       <c r="K51" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="L51" t="inlineStr">
         <is>
@@ -7593,22 +7593,22 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Valeria Correa</t>
+          <t>Julián Osorio</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>PRY-005</t>
+          <t>PRY-002</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Apto 991</t>
+          <t>Apto 719</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Paula Arenas</t>
+          <t>Sofía Prada</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -7617,16 +7617,16 @@
         </is>
       </c>
       <c r="G52" t="n">
-        <v>520000000</v>
+        <v>585000000</v>
       </c>
       <c r="H52" t="n">
         <v>1</v>
       </c>
       <c r="I52" s="27" t="n">
-        <v>45942</v>
+        <v>45935</v>
       </c>
       <c r="J52" s="27" t="n">
-        <v>45986</v>
+        <v>45979</v>
       </c>
       <c r="K52" t="n">
         <v>44</v>
@@ -7645,22 +7645,22 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Esteban Duque</t>
+          <t>Valeria Correa</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>PRY-005</t>
+          <t>PRY-003</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Apto 74</t>
+          <t>Apto 675</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Miguel Salazar</t>
+          <t>Sofía Prada</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -7669,16 +7669,16 @@
         </is>
       </c>
       <c r="G53" t="n">
-        <v>490000000</v>
+        <v>560000000</v>
       </c>
       <c r="H53" t="n">
         <v>1</v>
       </c>
       <c r="I53" s="27" t="n">
-        <v>45958</v>
+        <v>45925</v>
       </c>
       <c r="J53" s="27" t="n">
-        <v>46001</v>
+        <v>45968</v>
       </c>
       <c r="K53" t="n">
         <v>43</v>
@@ -7697,17 +7697,17 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Natalia Gaviria</t>
+          <t>Esteban Duque</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>PRY-006</t>
+          <t>PRY-003</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Apto 460</t>
+          <t>Apto 812</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -7721,16 +7721,16 @@
         </is>
       </c>
       <c r="G54" t="n">
-        <v>410000000</v>
+        <v>600000000</v>
       </c>
       <c r="H54" t="n">
         <v>1</v>
       </c>
       <c r="I54" s="27" t="n">
-        <v>45916</v>
+        <v>45950</v>
       </c>
       <c r="J54" s="27" t="n">
-        <v>45960</v>
+        <v>45994</v>
       </c>
       <c r="K54" t="n">
         <v>44</v>
@@ -7749,22 +7749,22 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Fabián Marín</t>
+          <t>Natalia Gaviria</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>PRY-006</t>
+          <t>PRY-005</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Apto 129</t>
+          <t>Apto 322</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Luis Bedoya</t>
+          <t>Sofía Prada</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -7773,16 +7773,16 @@
         </is>
       </c>
       <c r="G55" t="n">
-        <v>455000000</v>
+        <v>480000000</v>
       </c>
       <c r="H55" t="n">
         <v>1</v>
       </c>
       <c r="I55" s="27" t="n">
-        <v>45952</v>
+        <v>45910</v>
       </c>
       <c r="J55" s="27" t="n">
-        <v>45996</v>
+        <v>45954</v>
       </c>
       <c r="K55" t="n">
         <v>44</v>
@@ -7801,7 +7801,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Lorena Pineda</t>
+          <t>Fabián Marín</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -7825,16 +7825,16 @@
         </is>
       </c>
       <c r="G56" t="n">
-        <v>600000000</v>
+        <v>610000000</v>
       </c>
       <c r="H56" t="n">
         <v>1</v>
       </c>
       <c r="I56" s="27" t="n">
-        <v>45925</v>
+        <v>45945</v>
       </c>
       <c r="J56" s="27" t="n">
-        <v>45969</v>
+        <v>45989</v>
       </c>
       <c r="K56" t="n">
         <v>44</v>
@@ -7853,12 +7853,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Simón Vélez</t>
+          <t>Lorena Pineda</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>PRY-007</t>
+          <t>PRY-001</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -7868,7 +7868,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Paula Arenas</t>
+          <t>Ana Quintero</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -7877,19 +7877,19 @@
         </is>
       </c>
       <c r="G57" t="n">
-        <v>540000000</v>
+        <v>655000000</v>
       </c>
       <c r="H57" t="n">
         <v>1</v>
       </c>
       <c r="I57" s="27" t="n">
-        <v>45964</v>
+        <v>45912</v>
       </c>
       <c r="J57" s="27" t="n">
-        <v>46009</v>
+        <v>45956</v>
       </c>
       <c r="K57" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="L57" t="inlineStr">
         <is>
@@ -7897,17 +7897,578 @@
         </is>
       </c>
     </row>
-    <row r="58" ht="15.75" customHeight="1" s="25"/>
-    <row r="59" ht="15.75" customHeight="1" s="25"/>
-    <row r="60" ht="15.75" customHeight="1" s="25"/>
-    <row r="61" ht="15.75" customHeight="1" s="25"/>
-    <row r="62" ht="15.75" customHeight="1" s="25"/>
-    <row r="63" ht="15.75" customHeight="1" s="25"/>
-    <row r="64" ht="15.75" customHeight="1" s="25"/>
-    <row r="65" ht="15.75" customHeight="1" s="25"/>
-    <row r="66" ht="15.75" customHeight="1" s="25"/>
-    <row r="67" ht="15.75" customHeight="1" s="25"/>
-    <row r="68" ht="15.75" customHeight="1" s="25"/>
+    <row r="58" ht="15.75" customHeight="1" s="25">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>NEG-056</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Simón Vélez</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>PRY-003</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Apto 991</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Ana Quintero</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Ganado</t>
+        </is>
+      </c>
+      <c r="G58" t="n">
+        <v>520000000</v>
+      </c>
+      <c r="H58" t="n">
+        <v>1</v>
+      </c>
+      <c r="I58" s="27" t="n">
+        <v>45938</v>
+      </c>
+      <c r="J58" s="27" t="n">
+        <v>45982</v>
+      </c>
+      <c r="K58" t="n">
+        <v>44</v>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>Cierre exitoso Q4 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="15.75" customHeight="1" s="25">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>NEG-057</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Mariana Cifuentes</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>PRY-005</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Apto 74</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Ana Quintero</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Ganado</t>
+        </is>
+      </c>
+      <c r="G59" t="n">
+        <v>495000000</v>
+      </c>
+      <c r="H59" t="n">
+        <v>1</v>
+      </c>
+      <c r="I59" s="27" t="n">
+        <v>45918</v>
+      </c>
+      <c r="J59" s="27" t="n">
+        <v>45962</v>
+      </c>
+      <c r="K59" t="n">
+        <v>44</v>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>Cierre exitoso Q4 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="15.75" customHeight="1" s="25">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>NEG-058</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Daniela Ochoa</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>PRY-005</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Apto 129</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Ana Quintero</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Ganado</t>
+        </is>
+      </c>
+      <c r="G60" t="n">
+        <v>460000000</v>
+      </c>
+      <c r="H60" t="n">
+        <v>1</v>
+      </c>
+      <c r="I60" s="27" t="n">
+        <v>45952</v>
+      </c>
+      <c r="J60" s="27" t="n">
+        <v>45996</v>
+      </c>
+      <c r="K60" t="n">
+        <v>44</v>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>Cierre exitoso Q4 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="15.75" customHeight="1" s="25">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>NEG-059</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Sebastián Toro</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>PRY-006</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Apto 88</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Ana Quintero</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Ganado</t>
+        </is>
+      </c>
+      <c r="G61" t="n">
+        <v>430000000</v>
+      </c>
+      <c r="H61" t="n">
+        <v>1</v>
+      </c>
+      <c r="I61" s="27" t="n">
+        <v>45962</v>
+      </c>
+      <c r="J61" s="27" t="n">
+        <v>46005</v>
+      </c>
+      <c r="K61" t="n">
+        <v>43</v>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>Cierre exitoso Q4 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="15.75" customHeight="1" s="25">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>NEG-060</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Carolina Peláez</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>PRY-001</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Apto 246</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Miguel Salazar</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Ganado</t>
+        </is>
+      </c>
+      <c r="G62" t="n">
+        <v>720000000</v>
+      </c>
+      <c r="H62" t="n">
+        <v>1</v>
+      </c>
+      <c r="I62" s="27" t="n">
+        <v>45928</v>
+      </c>
+      <c r="J62" s="27" t="n">
+        <v>45971</v>
+      </c>
+      <c r="K62" t="n">
+        <v>43</v>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>Cierre exitoso Q4 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="15.75" customHeight="1" s="25">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>NEG-061</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Iván Montes</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>PRY-002</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Apto 133</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Miguel Salazar</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Ganado</t>
+        </is>
+      </c>
+      <c r="G63" t="n">
+        <v>600000000</v>
+      </c>
+      <c r="H63" t="n">
+        <v>1</v>
+      </c>
+      <c r="I63" s="27" t="n">
+        <v>45942</v>
+      </c>
+      <c r="J63" s="27" t="n">
+        <v>45986</v>
+      </c>
+      <c r="K63" t="n">
+        <v>44</v>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>Cierre exitoso Q4 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="15.75" customHeight="1" s="25">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>NEG-062</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Alejandra Ruiz</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>PRY-005</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Apto 517</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Miguel Salazar</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Ganado</t>
+        </is>
+      </c>
+      <c r="G64" t="n">
+        <v>470000000</v>
+      </c>
+      <c r="H64" t="n">
+        <v>1</v>
+      </c>
+      <c r="I64" s="27" t="n">
+        <v>45948</v>
+      </c>
+      <c r="J64" s="27" t="n">
+        <v>45992</v>
+      </c>
+      <c r="K64" t="n">
+        <v>44</v>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>Cierre exitoso Q4 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="15.75" customHeight="1" s="25">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>NEG-063</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Felipe Correa</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>PRY-007</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Apto 340</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Miguel Salazar</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Ganado</t>
+        </is>
+      </c>
+      <c r="G65" t="n">
+        <v>540000000</v>
+      </c>
+      <c r="H65" t="n">
+        <v>1</v>
+      </c>
+      <c r="I65" s="27" t="n">
+        <v>45963</v>
+      </c>
+      <c r="J65" s="27" t="n">
+        <v>46007</v>
+      </c>
+      <c r="K65" t="n">
+        <v>44</v>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>Cierre exitoso Q4 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="15.75" customHeight="1" s="25">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>NEG-064</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Gina Espinosa</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>PRY-003</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Apto 405</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Paula Arenas</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Ganado</t>
+        </is>
+      </c>
+      <c r="G66" t="n">
+        <v>570000000</v>
+      </c>
+      <c r="H66" t="n">
+        <v>1</v>
+      </c>
+      <c r="I66" s="27" t="n">
+        <v>45932</v>
+      </c>
+      <c r="J66" s="27" t="n">
+        <v>45975</v>
+      </c>
+      <c r="K66" t="n">
+        <v>43</v>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>Cierre exitoso Q4 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="15.75" customHeight="1" s="25">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>NEG-065</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Jorge Higuita</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>PRY-005</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Apto 233</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Paula Arenas</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Ganado</t>
+        </is>
+      </c>
+      <c r="G67" t="n">
+        <v>505000000</v>
+      </c>
+      <c r="H67" t="n">
+        <v>1</v>
+      </c>
+      <c r="I67" s="27" t="n">
+        <v>45955</v>
+      </c>
+      <c r="J67" s="27" t="n">
+        <v>45998</v>
+      </c>
+      <c r="K67" t="n">
+        <v>43</v>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>Cierre exitoso Q4 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="15.75" customHeight="1" s="25">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>NEG-066</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Manuela Franco</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>PRY-006</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Apto 512</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Paula Arenas</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Ganado</t>
+        </is>
+      </c>
+      <c r="G68" t="n">
+        <v>415000000</v>
+      </c>
+      <c r="H68" t="n">
+        <v>1</v>
+      </c>
+      <c r="I68" s="27" t="n">
+        <v>45969</v>
+      </c>
+      <c r="J68" s="27" t="n">
+        <v>46011</v>
+      </c>
+      <c r="K68" t="n">
+        <v>42</v>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>Cierre exitoso Q4 2025</t>
+        </is>
+      </c>
+    </row>
     <row r="69" ht="15.75" customHeight="1" s="25"/>
     <row r="70" ht="15.75" customHeight="1" s="25"/>
     <row r="71" ht="15.75" customHeight="1" s="25"/>
@@ -8856,7 +9417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K37"/>
+  <dimension ref="A1:K63"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="11" customWidth="1" style="25" min="1" max="1"/>
@@ -10651,32 +11212,1228 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="15.75" customHeight="1" s="25"/>
-    <row r="39" ht="15.75" customHeight="1" s="25"/>
-    <row r="40" ht="15.75" customHeight="1" s="25"/>
-    <row r="41" ht="15.75" customHeight="1" s="25"/>
-    <row r="42" ht="15.75" customHeight="1" s="25"/>
-    <row r="43" ht="15.75" customHeight="1" s="25"/>
-    <row r="44" ht="15.75" customHeight="1" s="25"/>
-    <row r="45" ht="15.75" customHeight="1" s="25"/>
-    <row r="46" ht="15.75" customHeight="1" s="25"/>
-    <row r="47" ht="15.75" customHeight="1" s="25"/>
-    <row r="48" ht="15.75" customHeight="1" s="25"/>
-    <row r="49" ht="15.75" customHeight="1" s="25"/>
-    <row r="50" ht="15.75" customHeight="1" s="25"/>
-    <row r="51" ht="15.75" customHeight="1" s="25"/>
-    <row r="52" ht="15.75" customHeight="1" s="25"/>
-    <row r="53" ht="15.75" customHeight="1" s="25"/>
-    <row r="54" ht="15.75" customHeight="1" s="25"/>
-    <row r="55" ht="15.75" customHeight="1" s="25"/>
-    <row r="56" ht="15.75" customHeight="1" s="25"/>
-    <row r="57" ht="15.75" customHeight="1" s="25"/>
-    <row r="58" ht="15.75" customHeight="1" s="25"/>
-    <row r="59" ht="15.75" customHeight="1" s="25"/>
-    <row r="60" ht="15.75" customHeight="1" s="25"/>
-    <row r="61" ht="15.75" customHeight="1" s="25"/>
-    <row r="62" ht="15.75" customHeight="1" s="25"/>
-    <row r="63" ht="15.75" customHeight="1" s="25"/>
+    <row r="38" ht="15.75" customHeight="1" s="25">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>PAG-036</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Diego Salcedo</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>PRY-001</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Separación</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>62000000</v>
+      </c>
+      <c r="F38" t="n">
+        <v>55000000</v>
+      </c>
+      <c r="G38" t="n">
+        <v>7000000</v>
+      </c>
+      <c r="H38" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="I38" s="27" t="n">
+        <v>45935</v>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Al día</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Luis Bedoya</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="15.75" customHeight="1" s="25">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>PAG-037</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Verónica Cárdenas</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>PRY-001</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Primera cuota</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>70000000</v>
+      </c>
+      <c r="F39" t="n">
+        <v>60000000</v>
+      </c>
+      <c r="G39" t="n">
+        <v>10000000</v>
+      </c>
+      <c r="H39" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="I39" s="27" t="n">
+        <v>45950</v>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Al día</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Luis Bedoya</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="15.75" customHeight="1" s="25">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>PAG-038</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Ricardo Palacio</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>PRY-001</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Separación</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>78000000</v>
+      </c>
+      <c r="F40" t="n">
+        <v>70000000</v>
+      </c>
+      <c r="G40" t="n">
+        <v>8000000</v>
+      </c>
+      <c r="H40" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="I40" s="27" t="n">
+        <v>45976</v>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Al día</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Luis Bedoya</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="15.75" customHeight="1" s="25">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>PAG-039</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Tomás Escobar</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>PRY-002</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Primera cuota</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>64000000</v>
+      </c>
+      <c r="F41" t="n">
+        <v>50000000</v>
+      </c>
+      <c r="G41" t="n">
+        <v>14000000</v>
+      </c>
+      <c r="H41" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="I41" s="27" t="n">
+        <v>45958</v>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Al día</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Luis Bedoya</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="15.75" customHeight="1" s="25">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>PAG-040</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Melissa Uribe</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>PRY-002</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Separación</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>59000000</v>
+      </c>
+      <c r="F42" t="n">
+        <v>45000000</v>
+      </c>
+      <c r="G42" t="n">
+        <v>14000000</v>
+      </c>
+      <c r="H42" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="I42" s="27" t="n">
+        <v>45983</v>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Luis Bedoya</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="15.75" customHeight="1" s="25">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>PAG-041</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Andrés Zuluaga</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>PRY-003</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Primera cuota</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>54000000</v>
+      </c>
+      <c r="F43" t="n">
+        <v>40000000</v>
+      </c>
+      <c r="G43" t="n">
+        <v>14000000</v>
+      </c>
+      <c r="H43" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="I43" s="27" t="n">
+        <v>45963</v>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Luis Bedoya</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="15.75" customHeight="1" s="25">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>PAG-042</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Paula Betancur</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>PRY-003</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Separación</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>61000000</v>
+      </c>
+      <c r="F44" t="n">
+        <v>50000000</v>
+      </c>
+      <c r="G44" t="n">
+        <v>11000000</v>
+      </c>
+      <c r="H44" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="I44" s="27" t="n">
+        <v>45999</v>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Al día</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Luis Bedoya</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="15.75" customHeight="1" s="25">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>PAG-043</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Camilo Restrepo</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>PRY-006</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Primera cuota</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>41000000</v>
+      </c>
+      <c r="F45" t="n">
+        <v>30000000</v>
+      </c>
+      <c r="G45" t="n">
+        <v>11000000</v>
+      </c>
+      <c r="H45" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="I45" s="27" t="n">
+        <v>46003</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Luis Bedoya</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="15.75" customHeight="1" s="25">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>PAG-044</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Sara Londoño</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>PRY-001</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Separación</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>69000000</v>
+      </c>
+      <c r="F46" t="n">
+        <v>60000000</v>
+      </c>
+      <c r="G46" t="n">
+        <v>9000000</v>
+      </c>
+      <c r="H46" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="I46" s="27" t="n">
+        <v>45944</v>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>Al día</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Sofía Prada</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="15.75" customHeight="1" s="25">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>PAG-045</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Julián Osorio</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>PRY-002</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Primera cuota</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>58000000</v>
+      </c>
+      <c r="F47" t="n">
+        <v>44000000</v>
+      </c>
+      <c r="G47" t="n">
+        <v>14000000</v>
+      </c>
+      <c r="H47" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="I47" s="27" t="n">
+        <v>45979</v>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Sofía Prada</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="15.75" customHeight="1" s="25">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>PAG-046</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Valeria Correa</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>PRY-003</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Separación</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>56000000</v>
+      </c>
+      <c r="F48" t="n">
+        <v>42000000</v>
+      </c>
+      <c r="G48" t="n">
+        <v>14000000</v>
+      </c>
+      <c r="H48" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="I48" s="27" t="n">
+        <v>45968</v>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Sofía Prada</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="15.75" customHeight="1" s="25">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>PAG-047</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Esteban Duque</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>PRY-003</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Primera cuota</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>60000000</v>
+      </c>
+      <c r="F49" t="n">
+        <v>48000000</v>
+      </c>
+      <c r="G49" t="n">
+        <v>12000000</v>
+      </c>
+      <c r="H49" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="I49" s="27" t="n">
+        <v>45994</v>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Al día</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Sofía Prada</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="15.75" customHeight="1" s="25">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>PAG-048</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Natalia Gaviria</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>PRY-005</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Separación</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>48000000</v>
+      </c>
+      <c r="F50" t="n">
+        <v>36000000</v>
+      </c>
+      <c r="G50" t="n">
+        <v>12000000</v>
+      </c>
+      <c r="H50" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="I50" s="27" t="n">
+        <v>45954</v>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>Al día</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Sofía Prada</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="15.75" customHeight="1" s="25">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>PAG-049</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Fabián Marín</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>PRY-007</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Primera cuota</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>61000000</v>
+      </c>
+      <c r="F51" t="n">
+        <v>48000000</v>
+      </c>
+      <c r="G51" t="n">
+        <v>13000000</v>
+      </c>
+      <c r="H51" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="I51" s="27" t="n">
+        <v>45989</v>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>Al día</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>Sofía Prada</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="15.75" customHeight="1" s="25">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>PAG-050</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Lorena Pineda</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>PRY-001</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Separación</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>65000000</v>
+      </c>
+      <c r="F52" t="n">
+        <v>58000000</v>
+      </c>
+      <c r="G52" t="n">
+        <v>7000000</v>
+      </c>
+      <c r="H52" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="I52" s="27" t="n">
+        <v>45956</v>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>Al día</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>Ana Quintero</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="15.75" customHeight="1" s="25">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>PAG-051</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Simón Vélez</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>PRY-003</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Primera cuota</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>52000000</v>
+      </c>
+      <c r="F53" t="n">
+        <v>38000000</v>
+      </c>
+      <c r="G53" t="n">
+        <v>14000000</v>
+      </c>
+      <c r="H53" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="I53" s="27" t="n">
+        <v>45982</v>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>Ana Quintero</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="15.75" customHeight="1" s="25">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>PAG-052</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Mariana Cifuentes</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>PRY-005</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Separación</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>49000000</v>
+      </c>
+      <c r="F54" t="n">
+        <v>36000000</v>
+      </c>
+      <c r="G54" t="n">
+        <v>13000000</v>
+      </c>
+      <c r="H54" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="I54" s="27" t="n">
+        <v>45962</v>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>Ana Quintero</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="15.75" customHeight="1" s="25">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>PAG-053</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Daniela Ochoa</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>PRY-005</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Primera cuota</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>46000000</v>
+      </c>
+      <c r="F55" t="n">
+        <v>33000000</v>
+      </c>
+      <c r="G55" t="n">
+        <v>13000000</v>
+      </c>
+      <c r="H55" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="I55" s="27" t="n">
+        <v>45996</v>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>Ana Quintero</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="15.75" customHeight="1" s="25">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>PAG-054</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Sebastián Toro</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>PRY-006</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Separación</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>43000000</v>
+      </c>
+      <c r="F56" t="n">
+        <v>30000000</v>
+      </c>
+      <c r="G56" t="n">
+        <v>13000000</v>
+      </c>
+      <c r="H56" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="I56" s="27" t="n">
+        <v>46005</v>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>Ana Quintero</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="15.75" customHeight="1" s="25">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>PAG-055</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Carolina Peláez</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>PRY-001</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Primera cuota</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>72000000</v>
+      </c>
+      <c r="F57" t="n">
+        <v>65000000</v>
+      </c>
+      <c r="G57" t="n">
+        <v>7000000</v>
+      </c>
+      <c r="H57" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="I57" s="27" t="n">
+        <v>45971</v>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>Al día</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>Miguel Salazar</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="15.75" customHeight="1" s="25">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>PAG-056</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Iván Montes</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>PRY-002</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Separación</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>60000000</v>
+      </c>
+      <c r="F58" t="n">
+        <v>46000000</v>
+      </c>
+      <c r="G58" t="n">
+        <v>14000000</v>
+      </c>
+      <c r="H58" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="I58" s="27" t="n">
+        <v>45986</v>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>Miguel Salazar</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="15.75" customHeight="1" s="25">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>PAG-057</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Alejandra Ruiz</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>PRY-005</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Primera cuota</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
+        <v>47000000</v>
+      </c>
+      <c r="F59" t="n">
+        <v>34000000</v>
+      </c>
+      <c r="G59" t="n">
+        <v>13000000</v>
+      </c>
+      <c r="H59" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="I59" s="27" t="n">
+        <v>45992</v>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>Miguel Salazar</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="15.75" customHeight="1" s="25">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>PAG-058</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Felipe Correa</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>PRY-007</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Separación</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>54000000</v>
+      </c>
+      <c r="F60" t="n">
+        <v>42000000</v>
+      </c>
+      <c r="G60" t="n">
+        <v>12000000</v>
+      </c>
+      <c r="H60" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="I60" s="27" t="n">
+        <v>46007</v>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>Al día</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>Miguel Salazar</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="15.75" customHeight="1" s="25">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>PAG-059</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Gina Espinosa</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>PRY-003</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Primera cuota</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>57000000</v>
+      </c>
+      <c r="F61" t="n">
+        <v>44000000</v>
+      </c>
+      <c r="G61" t="n">
+        <v>13000000</v>
+      </c>
+      <c r="H61" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="I61" s="27" t="n">
+        <v>45975</v>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>Al día</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>Paula Arenas</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="15.75" customHeight="1" s="25">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>PAG-060</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Jorge Higuita</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>PRY-005</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Separación</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>50500000</v>
+      </c>
+      <c r="F62" t="n">
+        <v>37000000</v>
+      </c>
+      <c r="G62" t="n">
+        <v>13500000</v>
+      </c>
+      <c r="H62" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="I62" s="27" t="n">
+        <v>45998</v>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>Paula Arenas</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="15.75" customHeight="1" s="25">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>PAG-061</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Manuela Franco</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>PRY-006</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Primera cuota</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
+        <v>42000000</v>
+      </c>
+      <c r="F63" t="n">
+        <v>29000000</v>
+      </c>
+      <c r="G63" t="n">
+        <v>13000000</v>
+      </c>
+      <c r="H63" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="I63" s="27" t="n">
+        <v>46011</v>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>Paula Arenas</t>
+        </is>
+      </c>
+    </row>
     <row r="64" ht="15.75" customHeight="1" s="25"/>
     <row r="65" ht="15.75" customHeight="1" s="25"/>
     <row r="66" ht="15.75" customHeight="1" s="25"/>

</xml_diff>